<commit_message>
Cape Verde for the draw!
</commit_message>
<xml_diff>
--- a/fasit/world_cup_2026_fasit.xlsx
+++ b/fasit/world_cup_2026_fasit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\hs\git\VM2026\fasit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0228E2A8-4687-468C-A561-6E8EC8F849A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD1E16B3-64B4-4CFF-8CD3-C8C0AEA41E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6120" yWindow="2910" windowWidth="28800" windowHeight="15345" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13157,12 +13157,56 @@
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -13243,50 +13287,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection hidden="1"/>
     </xf>
   </cellXfs>
@@ -40067,25 +40067,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:95" ht="46.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="139" t="str" cm="1">
+      <c r="A1" s="150" t="str" cm="1">
         <f t="array" ref="A1">INDEX(T,2,lang)</f>
         <v>2026 World Cup Final Tournament Schedule</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="139"/>
-      <c r="D1" s="139"/>
-      <c r="E1" s="139"/>
-      <c r="F1" s="139"/>
-      <c r="G1" s="139"/>
-      <c r="H1" s="139"/>
-      <c r="I1" s="139"/>
-      <c r="J1" s="139"/>
-      <c r="K1" s="139"/>
-      <c r="L1" s="139"/>
-      <c r="M1" s="139"/>
-      <c r="N1" s="139"/>
-      <c r="O1" s="139"/>
-      <c r="P1" s="139"/>
+      <c r="B1" s="150"/>
+      <c r="C1" s="150"/>
+      <c r="D1" s="150"/>
+      <c r="E1" s="150"/>
+      <c r="F1" s="150"/>
+      <c r="G1" s="150"/>
+      <c r="H1" s="150"/>
+      <c r="I1" s="150"/>
+      <c r="J1" s="150"/>
+      <c r="K1" s="150"/>
+      <c r="L1" s="150"/>
+      <c r="M1" s="150"/>
+      <c r="N1" s="150"/>
+      <c r="O1" s="150"/>
+      <c r="P1" s="150"/>
       <c r="S1" s="123"/>
       <c r="T1" s="123"/>
       <c r="AC1" s="123"/>
@@ -40132,11 +40132,11 @@
       <c r="L3" s="10"/>
       <c r="M3" s="10"/>
       <c r="N3" s="10"/>
-      <c r="O3" s="140" t="str">
+      <c r="O3" s="151" t="str">
         <f>"Language: " &amp; Settings!C4</f>
         <v>Language: English</v>
       </c>
-      <c r="P3" s="140"/>
+      <c r="P3" s="151"/>
       <c r="S3" s="123"/>
       <c r="T3" s="123"/>
       <c r="AC3" s="123"/>
@@ -40154,43 +40154,43 @@
     </row>
     <row r="4" spans="1:95" ht="3" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:95" x14ac:dyDescent="0.25">
-      <c r="A5" s="141" t="str" cm="1">
+      <c r="A5" s="152" t="str" cm="1">
         <f t="array" ref="A5">INDEX(T,3,lang)</f>
         <v>Group Stage</v>
       </c>
-      <c r="B5" s="142"/>
-      <c r="C5" s="142"/>
-      <c r="D5" s="142"/>
-      <c r="E5" s="142"/>
-      <c r="F5" s="142"/>
-      <c r="G5" s="142"/>
-      <c r="H5" s="143"/>
-      <c r="J5" s="147" t="s">
+      <c r="B5" s="153"/>
+      <c r="C5" s="153"/>
+      <c r="D5" s="153"/>
+      <c r="E5" s="153"/>
+      <c r="F5" s="153"/>
+      <c r="G5" s="153"/>
+      <c r="H5" s="154"/>
+      <c r="J5" s="158" t="s">
         <v>3166</v>
       </c>
-      <c r="K5" s="148"/>
-      <c r="L5" s="148"/>
-      <c r="M5" s="148"/>
-      <c r="N5" s="148"/>
-      <c r="O5" s="148"/>
-      <c r="P5" s="149"/>
+      <c r="K5" s="159"/>
+      <c r="L5" s="159"/>
+      <c r="M5" s="159"/>
+      <c r="N5" s="159"/>
+      <c r="O5" s="159"/>
+      <c r="P5" s="160"/>
     </row>
     <row r="6" spans="1:95" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="144"/>
-      <c r="B6" s="145"/>
-      <c r="C6" s="145"/>
-      <c r="D6" s="145"/>
-      <c r="E6" s="145"/>
-      <c r="F6" s="145"/>
-      <c r="G6" s="145"/>
-      <c r="H6" s="146"/>
-      <c r="J6" s="150"/>
-      <c r="K6" s="151"/>
-      <c r="L6" s="151"/>
-      <c r="M6" s="151"/>
-      <c r="N6" s="151"/>
-      <c r="O6" s="151"/>
-      <c r="P6" s="152"/>
+      <c r="A6" s="155"/>
+      <c r="B6" s="156"/>
+      <c r="C6" s="156"/>
+      <c r="D6" s="156"/>
+      <c r="E6" s="156"/>
+      <c r="F6" s="156"/>
+      <c r="G6" s="156"/>
+      <c r="H6" s="157"/>
+      <c r="J6" s="161"/>
+      <c r="K6" s="162"/>
+      <c r="L6" s="162"/>
+      <c r="M6" s="162"/>
+      <c r="N6" s="162"/>
+      <c r="O6" s="162"/>
+      <c r="P6" s="163"/>
       <c r="R6" s="123" t="s">
         <v>3167</v>
       </c>
@@ -40300,37 +40300,37 @@
       <c r="BI6" s="128" t="s">
         <v>3178</v>
       </c>
-      <c r="BK6" s="133" t="s">
+      <c r="BK6" s="144" t="s">
         <v>3179</v>
       </c>
-      <c r="BL6" s="134"/>
-      <c r="BM6" s="134"/>
-      <c r="BN6" s="134"/>
-      <c r="BO6" s="135"/>
-      <c r="BR6" s="133" t="str" cm="1">
+      <c r="BL6" s="145"/>
+      <c r="BM6" s="145"/>
+      <c r="BN6" s="145"/>
+      <c r="BO6" s="146"/>
+      <c r="BR6" s="144" t="str" cm="1">
         <f t="array" ref="BR6">INDEX(T,4,lang)</f>
         <v>Round of 16</v>
       </c>
-      <c r="BS6" s="134"/>
-      <c r="BT6" s="134"/>
-      <c r="BU6" s="134"/>
-      <c r="BV6" s="135"/>
-      <c r="BY6" s="133" t="str" cm="1">
+      <c r="BS6" s="145"/>
+      <c r="BT6" s="145"/>
+      <c r="BU6" s="145"/>
+      <c r="BV6" s="146"/>
+      <c r="BY6" s="144" t="str" cm="1">
         <f t="array" ref="BY6">INDEX(T,5,lang)</f>
         <v>Quarterfinals</v>
       </c>
-      <c r="BZ6" s="134"/>
-      <c r="CA6" s="134"/>
-      <c r="CB6" s="134"/>
-      <c r="CC6" s="135"/>
-      <c r="CF6" s="133" t="str" cm="1">
+      <c r="BZ6" s="145"/>
+      <c r="CA6" s="145"/>
+      <c r="CB6" s="145"/>
+      <c r="CC6" s="146"/>
+      <c r="CF6" s="144" t="str" cm="1">
         <f t="array" ref="CF6">INDEX(T,6,lang)</f>
         <v>Semi-Finals</v>
       </c>
-      <c r="CG6" s="134"/>
-      <c r="CH6" s="134"/>
-      <c r="CI6" s="134"/>
-      <c r="CJ6" s="135"/>
+      <c r="CG6" s="145"/>
+      <c r="CH6" s="145"/>
+      <c r="CI6" s="145"/>
+      <c r="CJ6" s="146"/>
     </row>
     <row r="7" spans="1:95" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11">
@@ -40407,26 +40407,26 @@
         <v>1</v>
       </c>
       <c r="AY7" s="126"/>
-      <c r="BK7" s="136"/>
-      <c r="BL7" s="137"/>
-      <c r="BM7" s="137"/>
-      <c r="BN7" s="137"/>
-      <c r="BO7" s="138"/>
-      <c r="BR7" s="136"/>
-      <c r="BS7" s="137"/>
-      <c r="BT7" s="137"/>
-      <c r="BU7" s="137"/>
-      <c r="BV7" s="138"/>
-      <c r="BY7" s="136"/>
-      <c r="BZ7" s="137"/>
-      <c r="CA7" s="137"/>
-      <c r="CB7" s="137"/>
-      <c r="CC7" s="138"/>
-      <c r="CF7" s="136"/>
-      <c r="CG7" s="137"/>
-      <c r="CH7" s="137"/>
-      <c r="CI7" s="137"/>
-      <c r="CJ7" s="138"/>
+      <c r="BK7" s="147"/>
+      <c r="BL7" s="148"/>
+      <c r="BM7" s="148"/>
+      <c r="BN7" s="148"/>
+      <c r="BO7" s="149"/>
+      <c r="BR7" s="147"/>
+      <c r="BS7" s="148"/>
+      <c r="BT7" s="148"/>
+      <c r="BU7" s="148"/>
+      <c r="BV7" s="149"/>
+      <c r="BY7" s="147"/>
+      <c r="BZ7" s="148"/>
+      <c r="CA7" s="148"/>
+      <c r="CB7" s="148"/>
+      <c r="CC7" s="149"/>
+      <c r="CF7" s="147"/>
+      <c r="CG7" s="148"/>
+      <c r="CH7" s="148"/>
+      <c r="CI7" s="148"/>
+      <c r="CJ7" s="149"/>
     </row>
     <row r="8" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A8" s="16">
@@ -41162,7 +41162,7 @@
         <f>BH10/BH12</f>
         <v>0</v>
       </c>
-      <c r="BK10" s="131">
+      <c r="BK10" s="141">
         <v>74</v>
       </c>
       <c r="BL10" s="24" t="str">
@@ -41425,7 +41425,7 @@
         <f>BH11/BH12</f>
         <v>0</v>
       </c>
-      <c r="BK11" s="132"/>
+      <c r="BK11" s="142"/>
       <c r="BL11" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!G3,AK80:AS91,9,FALSE),"3rd Group A/B/C/D/F")</f>
         <v>3rd Group A/B/C/D/F</v>
@@ -41663,7 +41663,7 @@
       <c r="BO12" s="21"/>
       <c r="BP12" s="114"/>
       <c r="BQ12" s="112"/>
-      <c r="BR12" s="131">
+      <c r="BR12" s="141">
         <v>89</v>
       </c>
       <c r="BS12" s="24" t="str">
@@ -41784,7 +41784,7 @@
         <v>46203.875</v>
       </c>
       <c r="BQ13" s="115"/>
-      <c r="BR13" s="132"/>
+      <c r="BR13" s="142"/>
       <c r="BS13" s="26" t="str">
         <f>IF(BP14&gt;BP15,BL14,IF(BP14&lt;BP15,BL15,""))</f>
         <v/>
@@ -42042,7 +42042,7 @@
         <f>BH14/BH18</f>
         <v>0.99019607843137258</v>
       </c>
-      <c r="BK14" s="131">
+      <c r="BK14" s="141">
         <v>77</v>
       </c>
       <c r="BL14" s="24" t="str">
@@ -42309,7 +42309,7 @@
         <f>BH15/BH18</f>
         <v>0.99019607843137258</v>
       </c>
-      <c r="BK15" s="132"/>
+      <c r="BK15" s="142"/>
       <c r="BL15" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!I3,AK80:AS91,9,FALSE),"3rd Group C/D/F/G/H")</f>
         <v>3rd Group C/D/F/G/H</v>
@@ -42583,7 +42583,7 @@
       <c r="BV16" s="21"/>
       <c r="BW16" s="114"/>
       <c r="BX16" s="112"/>
-      <c r="BY16" s="131">
+      <c r="BY16" s="141">
         <v>97</v>
       </c>
       <c r="BZ16" s="24" t="str">
@@ -42845,7 +42845,7 @@
       <c r="BV17" s="21"/>
       <c r="BW17" s="114"/>
       <c r="BX17" s="115"/>
-      <c r="BY17" s="132"/>
+      <c r="BY17" s="142"/>
       <c r="BZ17" s="26" t="str">
         <f>IF(BW20&gt;BW21,BS20,IF(BW20&lt;BW21,BS21,""))</f>
         <v/>
@@ -43049,7 +43049,7 @@
         <f>MAX(BH14:BH17)+1</f>
         <v>102</v>
       </c>
-      <c r="BK18" s="131">
+      <c r="BK18" s="141">
         <v>73</v>
       </c>
       <c r="BL18" s="24" t="str">
@@ -43153,7 +43153,7 @@
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="BK19" s="132"/>
+      <c r="BK19" s="142"/>
       <c r="BL19" s="26" t="str">
         <f>AS15</f>
         <v>2B</v>
@@ -43218,8 +43218,12 @@
         <f>AE50</f>
         <v>Spain</v>
       </c>
-      <c r="F20" s="19"/>
-      <c r="G20" s="20"/>
+      <c r="F20" s="19">
+        <v>0</v>
+      </c>
+      <c r="G20" s="20">
+        <v>0</v>
+      </c>
       <c r="H20" s="80" t="str">
         <f>AE51</f>
         <v>Cape Verde</v>
@@ -43258,15 +43262,15 @@
       </c>
       <c r="S20" s="127" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Spain_draw</v>
       </c>
       <c r="T20" s="127" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Cape Verde_draw</v>
       </c>
       <c r="U20" s="123">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V20" s="123">
         <f t="shared" si="3"/>
@@ -43278,7 +43282,7 @@
       </c>
       <c r="X20" s="123">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y20" s="123">
         <f t="shared" si="10"/>
@@ -43292,9 +43296,9 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AB20" s="123" t="str">
+      <c r="AB20" s="123">
         <f t="shared" si="6"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AD20" s="123">
         <f>COUNTIF(AR20:AR23,CONCATENATE("&gt;=",AR20))</f>
@@ -43427,7 +43431,7 @@
       <c r="BO20" s="21"/>
       <c r="BP20" s="114"/>
       <c r="BQ20" s="112"/>
-      <c r="BR20" s="131">
+      <c r="BR20" s="141">
         <v>90</v>
       </c>
       <c r="BS20" s="24" t="str">
@@ -43696,7 +43700,7 @@
         <v>46203.041666666672</v>
       </c>
       <c r="BQ21" s="115"/>
-      <c r="BR21" s="132"/>
+      <c r="BR21" s="142"/>
       <c r="BS21" s="26" t="str">
         <f>IF(BP22&gt;BP23,BL22,IF(BP22&lt;BP23,BL23,""))</f>
         <v/>
@@ -43946,7 +43950,7 @@
         <f>BH22/BH24</f>
         <v>0</v>
       </c>
-      <c r="BK22" s="131">
+      <c r="BK22" s="141">
         <v>75</v>
       </c>
       <c r="BL22" s="24" t="str">
@@ -44206,7 +44210,7 @@
         <f>BH23/BH24</f>
         <v>0</v>
       </c>
-      <c r="BK23" s="132"/>
+      <c r="BK23" s="142"/>
       <c r="BL23" s="26" t="str">
         <f>AS21</f>
         <v>2C</v>
@@ -44233,7 +44237,7 @@
       <c r="CC23" s="21"/>
       <c r="CD23" s="114"/>
       <c r="CE23" s="112"/>
-      <c r="CF23" s="131">
+      <c r="CF23" s="141">
         <v>101</v>
       </c>
       <c r="CG23" s="24" t="str">
@@ -44450,7 +44454,7 @@
       <c r="CC24" s="21"/>
       <c r="CD24" s="114"/>
       <c r="CE24" s="115"/>
-      <c r="CF24" s="132"/>
+      <c r="CF24" s="142"/>
       <c r="CG24" s="26" t="str">
         <f>IF(CD32&gt;CD33,BZ32,IF(CD32&lt;CD33,BZ33,""))</f>
         <v/>
@@ -44795,7 +44799,7 @@
         <f>BH26/BH30</f>
         <v>0</v>
       </c>
-      <c r="BK26" s="131">
+      <c r="BK26" s="141">
         <v>83</v>
       </c>
       <c r="BL26" s="24" t="str">
@@ -45059,7 +45063,7 @@
         <f>BH27/BH30</f>
         <v>0</v>
       </c>
-      <c r="BK27" s="132"/>
+      <c r="BK27" s="142"/>
       <c r="BL27" s="26" t="str">
         <f>AS75</f>
         <v>2L</v>
@@ -45330,7 +45334,7 @@
       <c r="BO28" s="21"/>
       <c r="BP28" s="114"/>
       <c r="BQ28" s="112"/>
-      <c r="BR28" s="131">
+      <c r="BR28" s="141">
         <v>93</v>
       </c>
       <c r="BS28" s="24" t="str">
@@ -45591,7 +45595,7 @@
         <v>46205.791666666672</v>
       </c>
       <c r="BQ29" s="115"/>
-      <c r="BR29" s="132"/>
+      <c r="BR29" s="142"/>
       <c r="BS29" s="26" t="str">
         <f>IF(BP30&gt;BP31,BL30,IF(BP30&lt;BP31,BL31,""))</f>
         <v/>
@@ -45801,7 +45805,7 @@
         <f>MAX(BH26:BH29)+1</f>
         <v>1</v>
       </c>
-      <c r="BK30" s="131">
+      <c r="BK30" s="141">
         <v>84</v>
       </c>
       <c r="BL30" s="24" t="str">
@@ -45908,7 +45912,7 @@
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="BK31" s="132"/>
+      <c r="BK31" s="142"/>
       <c r="BL31" s="26" t="str">
         <f>AS63</f>
         <v>2J</v>
@@ -46180,7 +46184,7 @@
       <c r="BV32" s="21"/>
       <c r="BW32" s="114"/>
       <c r="BX32" s="112"/>
-      <c r="BY32" s="131">
+      <c r="BY32" s="141">
         <v>98</v>
       </c>
       <c r="BZ32" s="24" t="str">
@@ -46440,7 +46444,7 @@
       <c r="BV33" s="21"/>
       <c r="BW33" s="114"/>
       <c r="BX33" s="115"/>
-      <c r="BY33" s="132"/>
+      <c r="BY33" s="142"/>
       <c r="BZ33" s="26" t="str">
         <f>IF(BW36&gt;BW37,BS36,IF(BW36&lt;BW37,BS37,""))</f>
         <v/>
@@ -46455,14 +46459,14 @@
       <c r="CE33" s="112"/>
       <c r="CK33" s="114"/>
       <c r="CL33" s="112"/>
-      <c r="CM33" s="133" t="str" cm="1">
+      <c r="CM33" s="144" t="str" cm="1">
         <f t="array" ref="CM33">INDEX(T,8,lang)</f>
         <v>Final</v>
       </c>
-      <c r="CN33" s="134"/>
-      <c r="CO33" s="134"/>
-      <c r="CP33" s="134"/>
-      <c r="CQ33" s="135"/>
+      <c r="CN33" s="145"/>
+      <c r="CO33" s="145"/>
+      <c r="CP33" s="145"/>
+      <c r="CQ33" s="146"/>
     </row>
     <row r="34" spans="1:96" x14ac:dyDescent="0.25">
       <c r="A34" s="16">
@@ -46682,7 +46686,7 @@
         <f>BH34/BH36</f>
         <v>0</v>
       </c>
-      <c r="BK34" s="131">
+      <c r="BK34" s="141">
         <v>81</v>
       </c>
       <c r="BL34" s="24" t="str">
@@ -46713,11 +46717,11 @@
       <c r="CE34" s="112"/>
       <c r="CK34" s="114"/>
       <c r="CL34" s="112"/>
-      <c r="CM34" s="136"/>
-      <c r="CN34" s="137"/>
-      <c r="CO34" s="137"/>
-      <c r="CP34" s="137"/>
-      <c r="CQ34" s="138"/>
+      <c r="CM34" s="147"/>
+      <c r="CN34" s="148"/>
+      <c r="CO34" s="148"/>
+      <c r="CP34" s="148"/>
+      <c r="CQ34" s="149"/>
     </row>
     <row r="35" spans="1:96" x14ac:dyDescent="0.25">
       <c r="A35" s="16">
@@ -46937,7 +46941,7 @@
         <f>BH35/BH36</f>
         <v>0</v>
       </c>
-      <c r="BK35" s="132"/>
+      <c r="BK35" s="142"/>
       <c r="BL35" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!F3,AK80:AS91,9,FALSE),"3rd Group B/E/F/I/J")</f>
         <v>3rd Group B/E/F/I/J</v>
@@ -47162,7 +47166,7 @@
       <c r="BO36" s="21"/>
       <c r="BP36" s="114"/>
       <c r="BQ36" s="112"/>
-      <c r="BR36" s="131">
+      <c r="BR36" s="141">
         <v>94</v>
       </c>
       <c r="BS36" s="24" t="str">
@@ -47282,7 +47286,7 @@
         <v>46204.833333333336</v>
       </c>
       <c r="BQ37" s="115"/>
-      <c r="BR37" s="132"/>
+      <c r="BR37" s="142"/>
       <c r="BS37" s="26" t="str">
         <f>IF(BP38&gt;BP39,BL38,IF(BP38&lt;BP39,BL39,""))</f>
         <v/>
@@ -47309,7 +47313,7 @@
       <c r="CJ37" s="21"/>
       <c r="CK37" s="114"/>
       <c r="CL37" s="112"/>
-      <c r="CM37" s="131">
+      <c r="CM37" s="141">
         <v>104</v>
       </c>
       <c r="CN37" s="24" t="str">
@@ -47546,7 +47550,7 @@
         <f>BH38/BH42</f>
         <v>0.98064516129032253</v>
       </c>
-      <c r="BK38" s="131">
+      <c r="BK38" s="141">
         <v>82</v>
       </c>
       <c r="BL38" s="24" t="str">
@@ -47576,7 +47580,7 @@
       <c r="CI38" s="21"/>
       <c r="CJ38" s="21"/>
       <c r="CL38" s="115"/>
-      <c r="CM38" s="132"/>
+      <c r="CM38" s="142"/>
       <c r="CN38" s="26" t="str">
         <f>IF(CK55&gt;CK56,CG55,IF(CK55&lt;CK56,CG56,""))</f>
         <v/>
@@ -47811,7 +47815,7 @@
         <f>BH39/BH42</f>
         <v>0.98064516129032253</v>
       </c>
-      <c r="BK39" s="132"/>
+      <c r="BK39" s="142"/>
       <c r="BL39" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!H3,AK80:AS91,9,FALSE),"3rd Group A/E/H/I/J")</f>
         <v>3rd Group A/E/H/I/J</v>
@@ -48487,7 +48491,7 @@
         <f>MAX(BH38:BH41)+1</f>
         <v>51.666666666666664</v>
       </c>
-      <c r="BK42" s="131">
+      <c r="BK42" s="141">
         <v>76</v>
       </c>
       <c r="BL42" s="24" t="str">
@@ -48580,7 +48584,7 @@
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="BK43" s="132"/>
+      <c r="BK43" s="142"/>
       <c r="BL43" s="26" t="str">
         <f>AS39</f>
         <v>2F</v>
@@ -48836,7 +48840,7 @@
       <c r="BO44" s="21"/>
       <c r="BP44" s="114"/>
       <c r="BQ44" s="112"/>
-      <c r="BR44" s="131">
+      <c r="BR44" s="141">
         <v>91</v>
       </c>
       <c r="BS44" s="24" t="str">
@@ -48851,14 +48855,14 @@
         <v/>
       </c>
       <c r="CK44" s="114"/>
-      <c r="CM44" s="133" t="str" cm="1">
+      <c r="CM44" s="144" t="str" cm="1">
         <f t="array" ref="CM44">INDEX(T,7,lang)</f>
         <v>Third-Place Play-Off</v>
       </c>
-      <c r="CN44" s="134"/>
-      <c r="CO44" s="134"/>
-      <c r="CP44" s="134"/>
-      <c r="CQ44" s="135"/>
+      <c r="CN44" s="145"/>
+      <c r="CO44" s="145"/>
+      <c r="CP44" s="145"/>
+      <c r="CQ44" s="146"/>
     </row>
     <row r="45" spans="1:96" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="16">
@@ -49095,7 +49099,7 @@
         <v>46203.708333333336</v>
       </c>
       <c r="BQ45" s="115"/>
-      <c r="BR45" s="132"/>
+      <c r="BR45" s="142"/>
       <c r="BS45" s="26" t="str">
         <f>IF(BP46&gt;BP47,BL46,IF(BP46&lt;BP47,BL47,""))</f>
         <v/>
@@ -49108,11 +49112,11 @@
         <v/>
       </c>
       <c r="CK45" s="114"/>
-      <c r="CM45" s="136"/>
-      <c r="CN45" s="137"/>
-      <c r="CO45" s="137"/>
-      <c r="CP45" s="137"/>
-      <c r="CQ45" s="138"/>
+      <c r="CM45" s="147"/>
+      <c r="CN45" s="148"/>
+      <c r="CO45" s="148"/>
+      <c r="CP45" s="148"/>
+      <c r="CQ45" s="149"/>
     </row>
     <row r="46" spans="1:96" x14ac:dyDescent="0.25">
       <c r="A46" s="16">
@@ -49332,7 +49336,7 @@
         <f>BH46/BH48</f>
         <v>0</v>
       </c>
-      <c r="BK46" s="131">
+      <c r="BK46" s="141">
         <v>78</v>
       </c>
       <c r="BL46" s="24" t="str">
@@ -49574,7 +49578,7 @@
         <f>BH47/BH48</f>
         <v>0</v>
       </c>
-      <c r="BK47" s="132"/>
+      <c r="BK47" s="142"/>
       <c r="BL47" s="26" t="str">
         <f>AS57</f>
         <v>2I</v>
@@ -49817,7 +49821,7 @@
       <c r="BV48" s="21"/>
       <c r="BW48" s="114"/>
       <c r="BX48" s="112"/>
-      <c r="BY48" s="131">
+      <c r="BY48" s="141">
         <v>99</v>
       </c>
       <c r="BZ48" s="24" t="str">
@@ -49833,7 +49837,7 @@
       </c>
       <c r="CK48" s="114"/>
       <c r="CL48" s="112"/>
-      <c r="CM48" s="131">
+      <c r="CM48" s="141">
         <v>103</v>
       </c>
       <c r="CN48" s="24" t="str">
@@ -49938,7 +49942,7 @@
       <c r="BV49" s="21"/>
       <c r="BW49" s="114"/>
       <c r="BX49" s="115"/>
-      <c r="BY49" s="132"/>
+      <c r="BY49" s="142"/>
       <c r="BZ49" s="26" t="str">
         <f>IF(BW52&gt;BW53,BS52,IF(BW52&lt;BW53,BS53,""))</f>
         <v/>
@@ -49952,7 +49956,7 @@
       </c>
       <c r="CK49" s="114"/>
       <c r="CL49" s="115"/>
-      <c r="CM49" s="132"/>
+      <c r="CM49" s="142"/>
       <c r="CN49" s="26" t="str">
         <f>IF(CK55&gt;CK56,CG56,IF(CK55&lt;CK56,CG55,""))</f>
         <v/>
@@ -50077,7 +50081,7 @@
       </c>
       <c r="AG50" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE50 &amp; "_draw")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH50" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE50 &amp; "_lose")</f>
@@ -50101,15 +50105,15 @@
       </c>
       <c r="AN50" s="123">
         <f>AF50*3+AG50</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO50" s="123">
         <f>AN50/AN54*10+BA50</f>
-        <v>0</v>
+        <v>5.9803921568627452</v>
       </c>
       <c r="AP50" s="123">
         <f>AO50*10000000+BI50*100+AM50/AM54*10+AI50/AI54*1++IF(AQ50=0,ROW(),AQ50)/2000000</f>
-        <v>9.3820000000000004E-4</v>
+        <v>59804019.608781338</v>
       </c>
       <c r="AQ50" s="126">
         <f>VLOOKUP(AE50,db_fifarank,2,FALSE)</f>
@@ -50117,7 +50121,7 @@
       </c>
       <c r="AR50" s="125">
         <f>AP50/AP54</f>
-        <v>9.3732060580763133E-4</v>
+        <v>0.9999999832787162</v>
       </c>
       <c r="AS50" s="125" t="str">
         <f>IF(SUM(AF50:AH53)=12,J51,"1H")</f>
@@ -50129,7 +50133,7 @@
       </c>
       <c r="AU50" s="126" cm="1">
         <f t="array" ref="AU50">SUMPRODUCT(($S$7:$S$78=AE50&amp;"_draw")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE50&amp;"_draw")*($U$7:$U$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV50" s="126" cm="1">
         <f t="array" ref="AV50">SUMPRODUCT(($E$7:$E$78=AE50)*($U$7:$U$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE50)*($U$7:$U$78)*($G$7:$G$78))</f>
@@ -50149,11 +50153,11 @@
       </c>
       <c r="AZ50" s="126">
         <f>AT50/AT54*1000+AU50/AU54*100+AY50/AY54*10+AV50/AV54</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="BA50" s="126">
         <f>AZ50/AZ54</f>
-        <v>0</v>
+        <v>0.98039215686274506</v>
       </c>
       <c r="BB50" s="126" cm="1">
         <f t="array" ref="BB50">SUMPRODUCT(($S$7:$S$78=AE50&amp;"_win")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE50&amp;"_win")*($X$7:$X$78))</f>
@@ -50161,7 +50165,7 @@
       </c>
       <c r="BC50" s="126" cm="1">
         <f t="array" ref="BC50">SUMPRODUCT(($S$7:$S$78=AE50&amp;"_draw")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE50&amp;"_draw")*($X$7:$X$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD50" s="126" cm="1">
         <f t="array" ref="BD50">SUMPRODUCT(($E$7:$E$78=AE50)*($X$7:$X$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE50)*($X$7:$X$78)*($G$7:$G$78))</f>
@@ -50181,13 +50185,13 @@
       </c>
       <c r="BH50" s="126">
         <f>BB50/BB54*1000+BC50/BC54*100+BG50/BG54*10+BD50/BD54</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="BI50" s="126">
         <f>BH50/BH54</f>
-        <v>0</v>
-      </c>
-      <c r="BK50" s="131">
+        <v>0.98039215686274506</v>
+      </c>
+      <c r="BK50" s="141">
         <v>79</v>
       </c>
       <c r="BL50" s="24" t="str">
@@ -50250,7 +50254,7 @@
       </c>
       <c r="K51" s="31">
         <f>L51+M51+N51</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" s="31">
         <f>VLOOKUP(1,AD50:AN53,3,FALSE)</f>
@@ -50258,7 +50262,7 @@
       </c>
       <c r="M51" s="31">
         <f>VLOOKUP(1,AD50:AN53,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N51" s="31">
         <f>VLOOKUP(1,AD50:AN53,5,FALSE)</f>
@@ -50270,7 +50274,7 @@
       </c>
       <c r="P51" s="32">
         <f>L51*3+M51</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R51" s="123">
         <f>DATE(2026,6,23)+TIME(9,0,0)+gmt_delta</f>
@@ -50318,7 +50322,7 @@
       </c>
       <c r="AD51" s="123">
         <f>COUNTIF(AR50:AR53,CONCATENATE("&gt;=",AR51))</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AE51" s="124" t="str">
         <f>VLOOKUP("Cape Verde",T,lang,FALSE)</f>
@@ -50330,7 +50334,7 @@
       </c>
       <c r="AG51" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE51 &amp; "_draw")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH51" s="123">
         <f>COUNTIF($S$7:$T$78,"=" &amp; AE51 &amp; "_lose")</f>
@@ -50354,15 +50358,15 @@
       </c>
       <c r="AN51" s="123">
         <f>AF51*3+AG51</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO51" s="123">
         <f>AN51/AN54*10+BA51</f>
-        <v>0</v>
+        <v>5.9803921568627452</v>
       </c>
       <c r="AP51" s="123">
         <f>AO51*10000000+BI51*100+AM51/AM54*10+AI51/AI54*1++IF(AQ51=0,ROW(),AQ51)/2000000</f>
-        <v>6.8306500000000006E-4</v>
+        <v>59804019.6085262</v>
       </c>
       <c r="AQ51" s="126">
         <f>VLOOKUP(AE51,db_fifarank,2,FALSE)</f>
@@ -50370,7 +50374,7 @@
       </c>
       <c r="AR51" s="125">
         <f>AP51/AP54</f>
-        <v>6.8242474910039407E-4</v>
+        <v>0.99999998327444994</v>
       </c>
       <c r="AS51" s="125" t="str">
         <f>IF(SUM(AF50:AH53)=12,J52,"2H")</f>
@@ -50382,7 +50386,7 @@
       </c>
       <c r="AU51" s="126" cm="1">
         <f t="array" ref="AU51">SUMPRODUCT(($S$7:$S$78=AE51&amp;"_draw")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE51&amp;"_draw")*($U$7:$U$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV51" s="126" cm="1">
         <f t="array" ref="AV51">SUMPRODUCT(($E$7:$E$78=AE51)*($U$7:$U$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE51)*($U$7:$U$78)*($G$7:$G$78))</f>
@@ -50402,11 +50406,11 @@
       </c>
       <c r="AZ51" s="126">
         <f>AT51/AT54*1000+AU51/AU54*100+AY51/AY54*10+AV51/AV54</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="BA51" s="126">
         <f>AZ51/AZ54</f>
-        <v>0</v>
+        <v>0.98039215686274506</v>
       </c>
       <c r="BB51" s="126" cm="1">
         <f t="array" ref="BB51">SUMPRODUCT(($S$7:$S$78=AE51&amp;"_win")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE51&amp;"_win")*($X$7:$X$78))</f>
@@ -50414,7 +50418,7 @@
       </c>
       <c r="BC51" s="126" cm="1">
         <f t="array" ref="BC51">SUMPRODUCT(($S$7:$S$78=AE51&amp;"_draw")*($X$7:$X$78))+SUMPRODUCT(($T$7:$T$78=AE51&amp;"_draw")*($X$7:$X$78))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD51" s="126" cm="1">
         <f t="array" ref="BD51">SUMPRODUCT(($E$7:$E$78=AE51)*($X$7:$X$78)*($F$7:$F$78))+SUMPRODUCT(($H$7:$H$78=AE51)*($X$7:$X$78)*($G$7:$G$78))</f>
@@ -50434,13 +50438,13 @@
       </c>
       <c r="BH51" s="126">
         <f>BB51/BB54*1000+BC51/BC54*100+BG51/BG54*10+BD51/BD54</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="BI51" s="126">
         <f>BH51/BH54</f>
-        <v>0</v>
-      </c>
-      <c r="BK51" s="132"/>
+        <v>0.98039215686274506</v>
+      </c>
+      <c r="BK51" s="142"/>
       <c r="BL51" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!D3,AK80:AS91,9,FALSE),"3rd Group C/E/F/H/I")</f>
         <v>3rd Group C/E/F/H/I</v>
@@ -50503,11 +50507,11 @@
       </c>
       <c r="J52" s="33" t="str">
         <f>VLOOKUP(2,AD50:AN53,2,FALSE)</f>
-        <v>Uruguay</v>
+        <v>Cape Verde</v>
       </c>
       <c r="K52" s="23">
         <f>L52+M52+N52</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L52" s="23">
         <f>VLOOKUP(2,AD50:AN53,3,FALSE)</f>
@@ -50515,7 +50519,7 @@
       </c>
       <c r="M52" s="23">
         <f>VLOOKUP(2,AD50:AN53,4,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N52" s="23">
         <f>VLOOKUP(2,AD50:AN53,5,FALSE)</f>
@@ -50527,7 +50531,7 @@
       </c>
       <c r="P52" s="34">
         <f>L52*3+M52</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R52" s="123">
         <f>DATE(2026,6,23)+TIME(12,0,0)+gmt_delta</f>
@@ -50575,7 +50579,7 @@
       </c>
       <c r="AD52" s="123">
         <f>COUNTIF(AR50:AR53,CONCATENATE("&gt;=",AR52))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE52" s="124" t="str">
         <f>VLOOKUP("Saudi Arabia",T,lang,FALSE)</f>
@@ -50627,7 +50631,7 @@
       </c>
       <c r="AR52" s="125">
         <f>AP52/AP54</f>
-        <v>7.1004883218564344E-4</v>
+        <v>1.1884067204264892E-11</v>
       </c>
       <c r="AT52" s="126" cm="1">
         <f t="array" ref="AT52">SUMPRODUCT(($S$7:$S$78=AE52&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE52&amp;"_win")*($U$7:$U$78))</f>
@@ -50700,7 +50704,7 @@
       <c r="BO52" s="21"/>
       <c r="BP52" s="114"/>
       <c r="BQ52" s="112"/>
-      <c r="BR52" s="131">
+      <c r="BR52" s="141">
         <v>92</v>
       </c>
       <c r="BS52" s="24" t="str">
@@ -50752,7 +50756,7 @@
       </c>
       <c r="J53" s="33" t="str">
         <f>VLOOKUP(3,AD50:AN53,2,FALSE)</f>
-        <v>Saudi Arabia</v>
+        <v>Uruguay</v>
       </c>
       <c r="K53" s="23">
         <f>L53+M53+N53</f>
@@ -50824,7 +50828,7 @@
       </c>
       <c r="AD53" s="123">
         <f>COUNTIF(AR50:AR53,CONCATENATE("&gt;=",AR53))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE53" s="124" t="str">
         <f>VLOOKUP("Uruguay",T,lang,FALSE)</f>
@@ -50876,7 +50880,7 @@
       </c>
       <c r="AR53" s="125">
         <f>AP53/AP54</f>
-        <v>8.3575089850702075E-4</v>
+        <v>1.3987939129918085E-11</v>
       </c>
       <c r="AT53" s="126" cm="1">
         <f t="array" ref="AT53">SUMPRODUCT(($S$7:$S$78=AE53&amp;"_win")*($U$7:$U$78))+SUMPRODUCT(($T$7:$T$78=AE53&amp;"_win")*($U$7:$U$78))</f>
@@ -50955,7 +50959,7 @@
         <v>46204.666666666672</v>
       </c>
       <c r="BQ53" s="115"/>
-      <c r="BR53" s="132"/>
+      <c r="BR53" s="142"/>
       <c r="BS53" s="26" t="str">
         <f>IF(BP54&gt;BP55,BL54,IF(BP54&lt;BP55,BL55,""))</f>
         <v/>
@@ -51005,7 +51009,7 @@
       </c>
       <c r="J54" s="35" t="str">
         <f>VLOOKUP(4,AD50:AN53,2,FALSE)</f>
-        <v>Cape Verde</v>
+        <v>Saudi Arabia</v>
       </c>
       <c r="K54" s="36">
         <f>L54+M54+N54</f>
@@ -51081,7 +51085,7 @@
       </c>
       <c r="AG54" s="123">
         <f t="shared" si="25"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH54" s="123">
         <f t="shared" si="25"/>
@@ -51101,15 +51105,15 @@
       </c>
       <c r="AN54" s="123">
         <f>MAX(AN50:AN53)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AO54" s="123">
         <f>MAX(AO50:AO53)+1</f>
-        <v>1</v>
+        <v>6.9803921568627452</v>
       </c>
       <c r="AP54" s="123">
         <f>MAX(AP50:AP53)+1</f>
-        <v>1.0009382</v>
+        <v>59804020.608781338</v>
       </c>
       <c r="AT54" s="126">
         <f>MAX(AT50:AT53)-MIN(AT50:AT53)+1</f>
@@ -51117,7 +51121,7 @@
       </c>
       <c r="AU54" s="126">
         <f>MAX(AU50:AU53)-MIN(AU50:AU53)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV54" s="126">
         <f>MAX(AV50:AV53)-MIN(AV50:AV53)+1</f>
@@ -51133,7 +51137,7 @@
       </c>
       <c r="AZ54" s="126">
         <f>MAX(AZ50:AZ53)+1</f>
-        <v>1</v>
+        <v>51</v>
       </c>
       <c r="BB54" s="126">
         <f>MAX(BB50:BB53)-MIN(BB50:BB53)+1</f>
@@ -51141,7 +51145,7 @@
       </c>
       <c r="BC54" s="126">
         <f>MAX(BC50:BC53)-MIN(BC50:BC53)+1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BD54" s="126">
         <f>MAX(BD50:BD53)-MIN(BD50:BD53)+1</f>
@@ -51157,9 +51161,9 @@
       </c>
       <c r="BH54" s="126">
         <f>MAX(BH50:BH53)+1</f>
-        <v>1</v>
-      </c>
-      <c r="BK54" s="131">
+        <v>51</v>
+      </c>
+      <c r="BK54" s="141">
         <v>80</v>
       </c>
       <c r="BL54" s="24" t="str">
@@ -51280,7 +51284,7 @@
         <f t="shared" si="23"/>
         <v/>
       </c>
-      <c r="BK55" s="132"/>
+      <c r="BK55" s="142"/>
       <c r="BL55" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!K3,AK80:AS91,9,FALSE),"3rd Group E/H/I/J/K")</f>
         <v>3rd Group E/H/I/J/K</v>
@@ -51307,7 +51311,7 @@
       <c r="CC55" s="21"/>
       <c r="CD55" s="114"/>
       <c r="CE55" s="112"/>
-      <c r="CF55" s="131">
+      <c r="CF55" s="141">
         <v>102</v>
       </c>
       <c r="CG55" s="24" t="str">
@@ -51566,7 +51570,7 @@
       <c r="CC56" s="21"/>
       <c r="CD56" s="114"/>
       <c r="CE56" s="115"/>
-      <c r="CF56" s="132"/>
+      <c r="CF56" s="142"/>
       <c r="CG56" s="26" t="str">
         <f>IF(CD64&gt;CD65,BZ64,IF(CD64&lt;CD65,BZ65,""))</f>
         <v/>
@@ -52049,7 +52053,7 @@
         <f>BH58/BH60</f>
         <v>0</v>
       </c>
-      <c r="BK58" s="131">
+      <c r="BK58" s="141">
         <v>86</v>
       </c>
       <c r="BL58" s="24" t="str">
@@ -52297,7 +52301,7 @@
         <f>BH59/BH60</f>
         <v>0</v>
       </c>
-      <c r="BK59" s="132"/>
+      <c r="BK59" s="142"/>
       <c r="BL59" s="26" t="str">
         <f>AS51</f>
         <v>2H</v>
@@ -52520,7 +52524,7 @@
       <c r="BO60" s="21"/>
       <c r="BP60" s="114"/>
       <c r="BQ60" s="112"/>
-      <c r="BR60" s="131">
+      <c r="BR60" s="141">
         <v>95</v>
       </c>
       <c r="BS60" s="24" t="str">
@@ -52633,7 +52637,7 @@
         <v>46206.75</v>
       </c>
       <c r="BQ61" s="115"/>
-      <c r="BR61" s="132"/>
+      <c r="BR61" s="142"/>
       <c r="BS61" s="26" t="str">
         <f>IF(BP62&gt;BP63,BL62,IF(BP62&lt;BP63,BL63,""))</f>
         <v/>
@@ -52876,7 +52880,7 @@
         <f>BH62/BH66</f>
         <v>0</v>
       </c>
-      <c r="BK62" s="131">
+      <c r="BK62" s="141">
         <v>88</v>
       </c>
       <c r="BL62" s="24" t="str">
@@ -53128,7 +53132,7 @@
         <f>BH63/BH66</f>
         <v>0</v>
       </c>
-      <c r="BK63" s="132"/>
+      <c r="BK63" s="142"/>
       <c r="BL63" s="26" t="str">
         <f>AS45</f>
         <v>2G</v>
@@ -53394,7 +53398,7 @@
       <c r="BV64" s="21"/>
       <c r="BW64" s="114"/>
       <c r="BX64" s="112"/>
-      <c r="BY64" s="131">
+      <c r="BY64" s="141">
         <v>100</v>
       </c>
       <c r="BZ64" s="24" t="str">
@@ -53648,7 +53652,7 @@
       <c r="BV65" s="21"/>
       <c r="BW65" s="114"/>
       <c r="BX65" s="115"/>
-      <c r="BY65" s="132"/>
+      <c r="BY65" s="142"/>
       <c r="BZ65" s="26" t="str">
         <f>IF(BW68&gt;BW69,BS68,IF(BW68&lt;BW69,BS69,""))</f>
         <v/>
@@ -53844,7 +53848,7 @@
         <f>MAX(BH62:BH65)+1</f>
         <v>1</v>
       </c>
-      <c r="BK66" s="131">
+      <c r="BK66" s="141">
         <v>85</v>
       </c>
       <c r="BL66" s="24" t="str">
@@ -53944,7 +53948,7 @@
         <f t="shared" si="23"/>
         <v/>
       </c>
-      <c r="BK67" s="132"/>
+      <c r="BK67" s="142"/>
       <c r="BL67" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!E3,AK80:AS91,9,FALSE),"3rd Group E/F/G/I/J")</f>
         <v>3rd Group E/F/G/I/J</v>
@@ -54200,7 +54204,7 @@
       <c r="BO68" s="21"/>
       <c r="BP68" s="114"/>
       <c r="BQ68" s="112"/>
-      <c r="BR68" s="131">
+      <c r="BR68" s="141">
         <v>96</v>
       </c>
       <c r="BS68" s="24" t="str">
@@ -54214,25 +54218,25 @@
         <f>IF(OR(BT68="",BT69="",AND(BU68="",BU69&lt;&gt;""),AND(BU69="",BU68&lt;&gt;""),AND(BV68="",BV69&lt;&gt;""),AND(BV69="",BV68&lt;&gt;"")),"",BT68*1000+BU68*10+BV68)</f>
         <v/>
       </c>
-      <c r="CE68" s="163" t="str">
+      <c r="CE68" s="143" t="str">
         <f>INDEX(T,144,lang)</f>
         <v>World Champion 2026</v>
       </c>
-      <c r="CF68" s="163"/>
-      <c r="CG68" s="163"/>
-      <c r="CH68" s="163"/>
-      <c r="CI68" s="163"/>
-      <c r="CJ68" s="163"/>
-      <c r="CK68" s="153" t="str">
+      <c r="CF68" s="143"/>
+      <c r="CG68" s="143"/>
+      <c r="CH68" s="143"/>
+      <c r="CI68" s="143"/>
+      <c r="CJ68" s="143"/>
+      <c r="CK68" s="131" t="str">
         <f>IF(CR37&gt;CR38,CN37,IF(CR37&lt;CR38,CN38,""))</f>
         <v/>
       </c>
-      <c r="CL68" s="153"/>
-      <c r="CM68" s="153"/>
-      <c r="CN68" s="153"/>
-      <c r="CO68" s="153"/>
-      <c r="CP68" s="153"/>
-      <c r="CQ68" s="153"/>
+      <c r="CL68" s="131"/>
+      <c r="CM68" s="131"/>
+      <c r="CN68" s="131"/>
+      <c r="CO68" s="131"/>
+      <c r="CP68" s="131"/>
+      <c r="CQ68" s="131"/>
     </row>
     <row r="69" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A69" s="16">
@@ -54470,7 +54474,7 @@
         <v>46207.0625</v>
       </c>
       <c r="BQ69" s="115"/>
-      <c r="BR69" s="132"/>
+      <c r="BR69" s="142"/>
       <c r="BS69" s="26" t="str">
         <f>IF(BP70&gt;BP71,BL70,IF(BP70&lt;BP71,BL71,""))</f>
         <v/>
@@ -54482,19 +54486,19 @@
         <f>IF(BW68="","",BT69*1000+BU69*10+BV69)</f>
         <v/>
       </c>
-      <c r="CE69" s="163"/>
-      <c r="CF69" s="163"/>
-      <c r="CG69" s="163"/>
-      <c r="CH69" s="163"/>
-      <c r="CI69" s="163"/>
-      <c r="CJ69" s="163"/>
-      <c r="CK69" s="153"/>
-      <c r="CL69" s="153"/>
-      <c r="CM69" s="153"/>
-      <c r="CN69" s="153"/>
-      <c r="CO69" s="153"/>
-      <c r="CP69" s="153"/>
-      <c r="CQ69" s="153"/>
+      <c r="CE69" s="143"/>
+      <c r="CF69" s="143"/>
+      <c r="CG69" s="143"/>
+      <c r="CH69" s="143"/>
+      <c r="CI69" s="143"/>
+      <c r="CJ69" s="143"/>
+      <c r="CK69" s="131"/>
+      <c r="CL69" s="131"/>
+      <c r="CM69" s="131"/>
+      <c r="CN69" s="131"/>
+      <c r="CO69" s="131"/>
+      <c r="CP69" s="131"/>
+      <c r="CQ69" s="131"/>
     </row>
     <row r="70" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A70" s="16">
@@ -54715,7 +54719,7 @@
         <f>BH70/BH72</f>
         <v>0</v>
       </c>
-      <c r="BK70" s="131">
+      <c r="BK70" s="141">
         <v>87</v>
       </c>
       <c r="BL70" s="24" t="str">
@@ -54951,7 +54955,7 @@
         <f>BH71/BH72</f>
         <v>0</v>
       </c>
-      <c r="BK71" s="132"/>
+      <c r="BK71" s="142"/>
       <c r="BL71" s="26" t="str">
         <f>IF(group_round_completed,VLOOKUP('3rd places'!J3,AK80:AS91,9,FALSE),"3rd Group D/E/I/J/L")</f>
         <v>3rd Group D/E/I/J/L</v>
@@ -56627,13 +56631,13 @@
     <row r="83" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="73"/>
       <c r="B83" s="73"/>
-      <c r="C83" s="154" t="s">
+      <c r="C83" s="132" t="s">
         <v>3183</v>
       </c>
-      <c r="D83" s="155"/>
-      <c r="E83" s="155"/>
-      <c r="F83" s="155"/>
-      <c r="G83" s="156"/>
+      <c r="D83" s="133"/>
+      <c r="E83" s="133"/>
+      <c r="F83" s="133"/>
+      <c r="G83" s="134"/>
       <c r="H83" s="75"/>
       <c r="I83" s="69"/>
       <c r="J83" s="99" t="str">
@@ -56731,16 +56735,16 @@
     <row r="84" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="73"/>
       <c r="B84" s="73"/>
-      <c r="C84" s="157"/>
-      <c r="D84" s="158"/>
-      <c r="E84" s="158"/>
-      <c r="F84" s="158"/>
-      <c r="G84" s="159"/>
+      <c r="C84" s="135"/>
+      <c r="D84" s="136"/>
+      <c r="E84" s="136"/>
+      <c r="F84" s="136"/>
+      <c r="G84" s="137"/>
       <c r="H84" s="75"/>
       <c r="I84" s="69"/>
       <c r="J84" s="99" t="str">
         <f>VLOOKUP(4,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓙ Algeria</v>
+        <v>Ⓗ Uruguay</v>
       </c>
       <c r="K84" s="100">
         <f t="shared" si="47"/>
@@ -56845,16 +56849,16 @@
     <row r="85" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="73"/>
       <c r="B85" s="73"/>
-      <c r="C85" s="157"/>
-      <c r="D85" s="158"/>
-      <c r="E85" s="158"/>
-      <c r="F85" s="158"/>
-      <c r="G85" s="159"/>
+      <c r="C85" s="135"/>
+      <c r="D85" s="136"/>
+      <c r="E85" s="136"/>
+      <c r="F85" s="136"/>
+      <c r="G85" s="137"/>
       <c r="H85" s="75"/>
       <c r="I85" s="69"/>
       <c r="J85" s="99" t="str">
         <f>VLOOKUP(5,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓖ Egypt</v>
+        <v>Ⓙ Algeria</v>
       </c>
       <c r="K85" s="100">
         <f t="shared" si="47"/>
@@ -56959,16 +56963,16 @@
     <row r="86" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="73"/>
       <c r="B86" s="73"/>
-      <c r="C86" s="157"/>
-      <c r="D86" s="158"/>
-      <c r="E86" s="158"/>
-      <c r="F86" s="158"/>
-      <c r="G86" s="159"/>
+      <c r="C86" s="135"/>
+      <c r="D86" s="136"/>
+      <c r="E86" s="136"/>
+      <c r="F86" s="136"/>
+      <c r="G86" s="137"/>
       <c r="H86" s="75"/>
       <c r="I86" s="69"/>
       <c r="J86" s="99" t="str">
         <f>VLOOKUP(6,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓘ Norway</v>
+        <v>Ⓖ Egypt</v>
       </c>
       <c r="K86" s="100">
         <f t="shared" si="47"/>
@@ -57008,7 +57012,7 @@
       </c>
       <c r="AD86" s="123">
         <f t="shared" si="38"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE86" s="124" t="str">
         <f>J47</f>
@@ -57073,16 +57077,16 @@
     <row r="87" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="73"/>
       <c r="B87" s="73"/>
-      <c r="C87" s="157"/>
-      <c r="D87" s="158"/>
-      <c r="E87" s="158"/>
-      <c r="F87" s="158"/>
-      <c r="G87" s="159"/>
+      <c r="C87" s="135"/>
+      <c r="D87" s="136"/>
+      <c r="E87" s="136"/>
+      <c r="F87" s="136"/>
+      <c r="G87" s="137"/>
       <c r="H87" s="75"/>
       <c r="I87" s="69"/>
       <c r="J87" s="99" t="str">
         <f>VLOOKUP(7,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓛ Panama</v>
+        <v>Ⓘ Norway</v>
       </c>
       <c r="K87" s="100">
         <f t="shared" si="47"/>
@@ -57122,11 +57126,11 @@
       </c>
       <c r="AD87" s="123">
         <f t="shared" si="38"/>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="AE87" s="124" t="str">
         <f>J53</f>
-        <v>Saudi Arabia</v>
+        <v>Uruguay</v>
       </c>
       <c r="AF87" s="123">
         <f t="shared" si="39"/>
@@ -57165,38 +57169,38 @@
       </c>
       <c r="AP87" s="123">
         <f>AN87/AN92*10000+AM87/AM92*1000+AI87/AI92*100+IF(AQ87=0,ROW(),AQ87)/2000000</f>
-        <v>666.6673773816666</v>
+        <v>666.66750320166659</v>
       </c>
       <c r="AQ87" s="126">
         <f t="shared" si="37"/>
-        <v>1421.43</v>
+        <v>1673.07</v>
       </c>
       <c r="AR87" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>BCFG</v>
+        <v>BCFGH</v>
       </c>
       <c r="AS87" s="129" t="str">
         <f t="shared" si="46"/>
-        <v/>
+        <v>Uruguay</v>
       </c>
       <c r="AT87" s="130" t="str">
         <f>"Ⓗ "&amp;AE87</f>
-        <v>Ⓗ Saudi Arabia</v>
+        <v>Ⓗ Uruguay</v>
       </c>
     </row>
     <row r="88" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="73"/>
       <c r="B88" s="73"/>
-      <c r="C88" s="160"/>
-      <c r="D88" s="161"/>
-      <c r="E88" s="161"/>
-      <c r="F88" s="161"/>
-      <c r="G88" s="162"/>
+      <c r="C88" s="138"/>
+      <c r="D88" s="139"/>
+      <c r="E88" s="139"/>
+      <c r="F88" s="139"/>
+      <c r="G88" s="140"/>
       <c r="H88" s="75"/>
       <c r="I88" s="69"/>
       <c r="J88" s="99" t="str">
         <f>VLOOKUP(8,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓚ DR Congo</v>
+        <v>Ⓛ Panama</v>
       </c>
       <c r="K88" s="100">
         <f t="shared" si="47"/>
@@ -57236,7 +57240,7 @@
       </c>
       <c r="AD88" s="123">
         <f t="shared" si="38"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AE88" s="124" t="str">
         <f>J59</f>
@@ -57287,7 +57291,7 @@
       </c>
       <c r="AR88" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>BCFGI</v>
+        <v>BCFGHI</v>
       </c>
       <c r="AS88" s="129" t="str">
         <f t="shared" si="46"/>
@@ -57310,7 +57314,7 @@
       <c r="I89" s="69"/>
       <c r="J89" s="102" t="str">
         <f>VLOOKUP(9,$AD$80:$AT$91,17,FALSE)</f>
-        <v>Ⓗ Saudi Arabia</v>
+        <v>Ⓚ DR Congo</v>
       </c>
       <c r="K89" s="103">
         <f t="shared" si="47"/>
@@ -57350,7 +57354,7 @@
       </c>
       <c r="AD89" s="123">
         <f t="shared" si="38"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AE89" s="124" t="str">
         <f>J65</f>
@@ -57401,7 +57405,7 @@
       </c>
       <c r="AR89" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>BCFGIJ</v>
+        <v>BCFGHIJ</v>
       </c>
       <c r="AS89" s="129" t="str">
         <f t="shared" si="46"/>
@@ -57464,7 +57468,7 @@
       </c>
       <c r="AD90" s="123">
         <f t="shared" si="38"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AE90" s="124" t="str">
         <f>J71</f>
@@ -57515,11 +57519,11 @@
       </c>
       <c r="AR90" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>BCFGIJK</v>
+        <v>BCFGHIJ</v>
       </c>
       <c r="AS90" s="129" t="str">
         <f t="shared" si="46"/>
-        <v>DR Congo</v>
+        <v/>
       </c>
       <c r="AT90" s="130" t="str">
         <f>"Ⓚ "&amp;AE90</f>
@@ -57578,7 +57582,7 @@
       </c>
       <c r="AD91" s="123">
         <f t="shared" si="38"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AE91" s="124" t="str">
         <f>J77</f>
@@ -57629,7 +57633,7 @@
       </c>
       <c r="AR91" s="125" t="str">
         <f t="shared" si="50"/>
-        <v>BCFGIJKL</v>
+        <v>BCFGHIJL</v>
       </c>
       <c r="AS91" s="129" t="str">
         <f t="shared" si="46"/>
@@ -57868,6 +57872,36 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="7nWuIQAsd0NKRlhwUK3tOeNHpTch5B5FULy2gxNNaIdJM5RfhFSMzPcx55y+pmM3d73guUy+p5Y+SvIjJZQRaA==" saltValue="Uw23KnM8csnTioq5H8upCA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="45">
+    <mergeCell ref="BK14:BK15"/>
+    <mergeCell ref="BY16:BY17"/>
+    <mergeCell ref="BK26:BK27"/>
+    <mergeCell ref="BR28:BR29"/>
+    <mergeCell ref="BK22:BK23"/>
+    <mergeCell ref="CF23:CF24"/>
+    <mergeCell ref="BK18:BK19"/>
+    <mergeCell ref="BR20:BR21"/>
+    <mergeCell ref="CM48:CM49"/>
+    <mergeCell ref="BR44:BR45"/>
+    <mergeCell ref="BK46:BK47"/>
+    <mergeCell ref="BK30:BK31"/>
+    <mergeCell ref="CM44:CQ45"/>
+    <mergeCell ref="BY32:BY33"/>
+    <mergeCell ref="BK38:BK39"/>
+    <mergeCell ref="BK34:BK35"/>
+    <mergeCell ref="BR36:BR37"/>
+    <mergeCell ref="BK42:BK43"/>
+    <mergeCell ref="CM33:CQ34"/>
+    <mergeCell ref="CM37:CM38"/>
+    <mergeCell ref="BK10:BK11"/>
+    <mergeCell ref="BR12:BR13"/>
+    <mergeCell ref="BK6:BO7"/>
+    <mergeCell ref="BR6:BV7"/>
+    <mergeCell ref="BY6:CC7"/>
+    <mergeCell ref="CF6:CJ7"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="A5:H6"/>
+    <mergeCell ref="J5:P6"/>
     <mergeCell ref="CK68:CQ69"/>
     <mergeCell ref="C83:G88"/>
     <mergeCell ref="BK70:BK71"/>
@@ -57883,36 +57917,6 @@
     <mergeCell ref="BR52:BR53"/>
     <mergeCell ref="BK54:BK55"/>
     <mergeCell ref="CE68:CJ69"/>
-    <mergeCell ref="CF6:CJ7"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="A5:H6"/>
-    <mergeCell ref="J5:P6"/>
-    <mergeCell ref="BK10:BK11"/>
-    <mergeCell ref="BR12:BR13"/>
-    <mergeCell ref="BK6:BO7"/>
-    <mergeCell ref="BR6:BV7"/>
-    <mergeCell ref="BY6:CC7"/>
-    <mergeCell ref="CF23:CF24"/>
-    <mergeCell ref="BK18:BK19"/>
-    <mergeCell ref="BR20:BR21"/>
-    <mergeCell ref="CM48:CM49"/>
-    <mergeCell ref="BR44:BR45"/>
-    <mergeCell ref="BK46:BK47"/>
-    <mergeCell ref="BK30:BK31"/>
-    <mergeCell ref="CM44:CQ45"/>
-    <mergeCell ref="BY32:BY33"/>
-    <mergeCell ref="BK38:BK39"/>
-    <mergeCell ref="BK34:BK35"/>
-    <mergeCell ref="BR36:BR37"/>
-    <mergeCell ref="BK42:BK43"/>
-    <mergeCell ref="CM33:CQ34"/>
-    <mergeCell ref="CM37:CM38"/>
-    <mergeCell ref="BK14:BK15"/>
-    <mergeCell ref="BY16:BY17"/>
-    <mergeCell ref="BK26:BK27"/>
-    <mergeCell ref="BR28:BR29"/>
-    <mergeCell ref="BK22:BK23"/>
   </mergeCells>
   <conditionalFormatting sqref="A7:E78">
     <cfRule type="expression" dxfId="228" priority="339">
@@ -58955,15 +58959,15 @@
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="109">
         <f>MATCH(C3,C6:C500,0)</f>
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C3" s="121" t="str">
         <f>'2026 World Cup'!AR91</f>
-        <v>BCFGIJKL</v>
+        <v>BCFGHIJL</v>
       </c>
       <c r="D3" s="121" t="str">
         <f>VLOOKUP($C3,$C$6:$K$500,2,FALSE)</f>
-        <v>3I</v>
+        <v>3H</v>
       </c>
       <c r="E3" s="121" t="str">
         <f>VLOOKUP($C3,$C$6:$K$500,3,FALSE)</f>
@@ -58991,7 +58995,7 @@
       </c>
       <c r="K3" s="122" t="str">
         <f>VLOOKUP($C3,$C$6:$K$500,9,FALSE)</f>
-        <v>3K</v>
+        <v>3I</v>
       </c>
     </row>
     <row r="5" spans="2:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>